<commit_message>
Portfolio V2 dashboard and import automation
</commit_message>
<xml_diff>
--- a/excel/Afranga.xlsx
+++ b/excel/Afranga.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Investavimas 2026.06.03\Afranga\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-v2\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77CB66F3-030C-406A-B6C0-AAA73EAB2672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECD71F8C-0C73-4DB7-8184-D9BDDC488DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="K3" s="17">
         <f ca="1">'10000159'!B12</f>
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="L3" s="17" t="str">
         <f ca="1">'10000159'!P3</f>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="T3" s="32">
         <f>W3-R3</f>
-        <v>0.92000000000001592</v>
+        <v>1.5300000000000296</v>
       </c>
       <c r="U3" s="32">
         <f>SUM(M3:M100)</f>
@@ -1990,27 +1990,27 @@
       </c>
       <c r="V3" s="32">
         <f>SUM(N3:N100)-AA3</f>
-        <v>12.519999999999998</v>
+        <v>13.130000000000003</v>
       </c>
       <c r="W3" s="32">
         <f>Q3+V3+S3</f>
-        <v>304.39</v>
+        <v>305</v>
       </c>
       <c r="X3" s="32">
         <f>W3-Q3</f>
-        <v>14.389999999999986</v>
+        <v>15</v>
       </c>
       <c r="Y3" s="35">
         <f>(W3-Q3)/Q3</f>
-        <v>4.9620689655172363E-2</v>
+        <v>5.1724137931034482E-2</v>
       </c>
       <c r="Z3" s="35">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>9.4052109122276323E-2</v>
+        <v>9.5573046803474435E-2</v>
       </c>
       <c r="AA3" s="32">
         <f>SUM(O3:O100)</f>
-        <v>1.4600000000000002</v>
+        <v>1.5300000000000002</v>
       </c>
       <c r="AC3" s="3" t="str">
         <f ca="1">'10000159'!Z3</f>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="K4" s="17">
         <f ca="1">'10000160'!B12</f>
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="L4" s="17" t="str">
         <f ca="1">'10000160'!P3</f>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="K5" s="17">
         <f ca="1">'10000158'!B12</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L5" s="17" t="str">
         <f ca="1">'10000158'!P3</f>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="K6" s="17">
         <f ca="1">'10000170'!B12</f>
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="L6" s="17" t="str">
         <f ca="1">'10000170'!P3</f>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="K7" s="17">
         <f ca="1">'10000212'!B12</f>
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="L7" s="17" t="str">
         <f ca="1">'10000212'!P3</f>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="K8" s="17">
         <f ca="1">'10000263'!B12</f>
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="L8" s="17" t="str">
         <f ca="1">'10000263'!P3</f>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="K9" s="17">
         <f ca="1">'10000288'!B12</f>
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="L9" s="17" t="str">
         <f ca="1">'10000288'!P3</f>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="K10" s="17">
         <f ca="1">'10000437'!B12</f>
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="L10" s="17" t="str">
         <f ca="1">'10000437'!P3</f>
@@ -2478,11 +2478,11 @@
       </c>
       <c r="N10" s="3">
         <f>'10000437'!L3</f>
-        <v>0.94</v>
+        <v>1.23</v>
       </c>
       <c r="O10" s="3">
         <f>'10000437'!M3</f>
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="P10" s="9"/>
       <c r="AC10" s="3" t="str">
@@ -2532,7 +2532,7 @@
       </c>
       <c r="K11" s="17">
         <f ca="1">'10000591'!B12</f>
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="L11" s="17" t="str">
         <f ca="1">'10000591'!P3</f>
@@ -2544,11 +2544,11 @@
       </c>
       <c r="N11" s="3">
         <f>'10000591'!L3</f>
-        <v>0.45</v>
+        <v>0.66</v>
       </c>
       <c r="O11" s="3">
         <f>'10000591'!M3</f>
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="P11" s="9"/>
       <c r="AC11" s="3" t="str">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="K12" s="17">
         <f ca="1">'10000722'!B12</f>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="L12" s="17" t="str">
         <f ca="1">'10000722'!P3</f>
@@ -2610,11 +2610,11 @@
       </c>
       <c r="N12" s="3">
         <f>'10000722'!L3</f>
-        <v>0.2</v>
+        <v>0.38</v>
       </c>
       <c r="O12" s="3">
         <f>'10000722'!M3</f>
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="P12" s="9"/>
       <c r="AC12" s="3" t="str">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="K13" s="17">
         <f ca="1">'10001244'!B12</f>
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="L13" s="17" t="str">
         <f ca="1">'10001244'!P3</f>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -4827,7 +4827,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -7531,7 +7531,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -10013,14 +10013,14 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="6">
         <f ca="1">TODAY()</f>
-        <v>46227</v>
+        <v>46232</v>
       </c>
       <c r="B200" s="1"/>
       <c r="C200" s="1"/>
       <c r="D200" s="1"/>
       <c r="K200" s="28">
         <f>Overview!W3</f>
-        <v>304.39</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -11438,11 +11438,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.2</v>
+        <v>0.38</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -11481,12 +11481,25 @@
       <c r="B4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="D4" s="10">
+        <v>46231</v>
+      </c>
+      <c r="E4" s="10">
+        <v>46231</v>
+      </c>
+      <c r="F4" s="17">
+        <f t="shared" ref="F4:F10" si="0">IF(E4&gt;0,E4-D4,"")</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0.18</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0.02</v>
+      </c>
       <c r="J4" s="9"/>
       <c r="X4" s="6">
         <f>E3</f>
@@ -11503,7 +11516,7 @@
       <c r="D5" s="10"/>
       <c r="E5" s="10"/>
       <c r="F5" s="17" t="str">
-        <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="G5" s="3"/>
@@ -11512,11 +11525,11 @@
       <c r="J5" s="9"/>
       <c r="X5" s="6">
         <f t="shared" ref="X5:X52" si="1">E4</f>
-        <v>0</v>
+        <v>46231</v>
       </c>
       <c r="Y5" s="3">
         <f t="shared" ref="Y5:Y52" si="2">G4+H4-I4</f>
-        <v>0</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
@@ -11652,7 +11665,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="6"/>
       <c r="F11" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F11:F52" si="3">IF(E11&gt;0,E11-D11,"")</f>
         <v/>
       </c>
       <c r="G11" s="2"/>
@@ -11674,12 +11687,12 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
       <c r="F12" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G12" s="2"/>
@@ -11701,7 +11714,7 @@
       <c r="D13" s="10"/>
       <c r="E13" s="6"/>
       <c r="F13" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G13" s="2"/>
@@ -11724,7 +11737,7 @@
       <c r="D14" s="10"/>
       <c r="E14" s="6"/>
       <c r="F14" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G14" s="2"/>
@@ -11750,7 +11763,7 @@
       <c r="D15" s="10"/>
       <c r="E15" s="6"/>
       <c r="F15" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G15" s="2"/>
@@ -11783,7 +11796,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="6"/>
       <c r="F16" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G16" s="2"/>
@@ -11810,7 +11823,7 @@
       <c r="D17" s="10"/>
       <c r="E17" s="6"/>
       <c r="F17" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G17" s="2"/>
@@ -11830,7 +11843,7 @@
       <c r="D18" s="10"/>
       <c r="E18" s="6"/>
       <c r="F18" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G18" s="2"/>
@@ -11850,7 +11863,7 @@
       <c r="D19" s="10"/>
       <c r="E19" s="6"/>
       <c r="F19" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G19" s="2"/>
@@ -11870,7 +11883,7 @@
       <c r="D20" s="10"/>
       <c r="E20" s="6"/>
       <c r="F20" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G20" s="2"/>
@@ -11890,7 +11903,7 @@
       <c r="D21" s="10"/>
       <c r="E21" s="6"/>
       <c r="F21" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G21" s="2"/>
@@ -11910,7 +11923,7 @@
       <c r="D22" s="10"/>
       <c r="E22" s="6"/>
       <c r="F22" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G22" s="2"/>
@@ -11930,7 +11943,7 @@
       <c r="D23" s="10"/>
       <c r="E23" s="6"/>
       <c r="F23" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G23" s="2"/>
@@ -11950,7 +11963,7 @@
       <c r="D24" s="10"/>
       <c r="E24" s="6"/>
       <c r="F24" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G24" s="2"/>
@@ -11970,7 +11983,7 @@
       <c r="D25" s="10"/>
       <c r="E25" s="6"/>
       <c r="F25" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G25" s="2"/>
@@ -11990,7 +12003,7 @@
       <c r="D26" s="10"/>
       <c r="E26" s="6"/>
       <c r="F26" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G26" s="2"/>
@@ -12010,7 +12023,7 @@
       <c r="D27" s="10"/>
       <c r="E27" s="6"/>
       <c r="F27" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G27" s="2"/>
@@ -12030,7 +12043,7 @@
       <c r="D28" s="10"/>
       <c r="E28" s="6"/>
       <c r="F28" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G28" s="2"/>
@@ -12050,7 +12063,7 @@
       <c r="D29" s="10"/>
       <c r="E29" s="6"/>
       <c r="F29" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G29" s="2"/>
@@ -12070,7 +12083,7 @@
       <c r="D30" s="10"/>
       <c r="E30" s="6"/>
       <c r="F30" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G30" s="2"/>
@@ -12090,7 +12103,7 @@
       <c r="D31" s="10"/>
       <c r="E31" s="6"/>
       <c r="F31" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G31" s="2"/>
@@ -12110,7 +12123,7 @@
       <c r="D32" s="10"/>
       <c r="E32" s="6"/>
       <c r="F32" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G32" s="2"/>
@@ -12130,7 +12143,7 @@
       <c r="D33" s="10"/>
       <c r="E33" s="6"/>
       <c r="F33" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G33" s="2"/>
@@ -12150,7 +12163,7 @@
       <c r="D34" s="10"/>
       <c r="E34" s="6"/>
       <c r="F34" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G34" s="2"/>
@@ -12170,7 +12183,7 @@
       <c r="D35" s="10"/>
       <c r="E35" s="6"/>
       <c r="F35" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G35" s="2"/>
@@ -12190,7 +12203,7 @@
       <c r="D36" s="10"/>
       <c r="E36" s="6"/>
       <c r="F36" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G36" s="2"/>
@@ -12210,7 +12223,7 @@
       <c r="D37" s="10"/>
       <c r="E37" s="6"/>
       <c r="F37" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G37" s="2"/>
@@ -12230,7 +12243,7 @@
       <c r="D38" s="10"/>
       <c r="E38" s="6"/>
       <c r="F38" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G38" s="2"/>
@@ -12250,7 +12263,7 @@
       <c r="D39" s="10"/>
       <c r="E39" s="6"/>
       <c r="F39" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G39" s="2"/>
@@ -12270,7 +12283,7 @@
       <c r="D40" s="10"/>
       <c r="E40" s="6"/>
       <c r="F40" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G40" s="2"/>
@@ -12290,7 +12303,7 @@
       <c r="D41" s="10"/>
       <c r="E41" s="6"/>
       <c r="F41" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G41" s="2"/>
@@ -12310,7 +12323,7 @@
       <c r="D42" s="10"/>
       <c r="E42" s="6"/>
       <c r="F42" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G42" s="2"/>
@@ -12330,7 +12343,7 @@
       <c r="D43" s="10"/>
       <c r="E43" s="6"/>
       <c r="F43" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G43" s="2"/>
@@ -12350,7 +12363,7 @@
       <c r="D44" s="10"/>
       <c r="E44" s="6"/>
       <c r="F44" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G44" s="2"/>
@@ -12370,7 +12383,7 @@
       <c r="D45" s="10"/>
       <c r="E45" s="6"/>
       <c r="F45" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G45" s="2"/>
@@ -12390,7 +12403,7 @@
       <c r="D46" s="10"/>
       <c r="E46" s="6"/>
       <c r="F46" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G46" s="2"/>
@@ -12410,7 +12423,7 @@
       <c r="D47" s="10"/>
       <c r="E47" s="6"/>
       <c r="F47" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G47" s="2"/>
@@ -12430,7 +12443,7 @@
       <c r="D48" s="10"/>
       <c r="E48" s="6"/>
       <c r="F48" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G48" s="2"/>
@@ -12450,7 +12463,7 @@
       <c r="D49" s="10"/>
       <c r="E49" s="6"/>
       <c r="F49" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G49" s="2"/>
@@ -12470,7 +12483,7 @@
       <c r="D50" s="10"/>
       <c r="E50" s="6"/>
       <c r="F50" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G50" s="2"/>
@@ -12490,7 +12503,7 @@
       <c r="D51" s="10"/>
       <c r="E51" s="6"/>
       <c r="F51" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G51" s="2"/>
@@ -12510,7 +12523,7 @@
       <c r="D52" s="10"/>
       <c r="E52" s="6"/>
       <c r="F52" s="17" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
       <c r="G52" s="2"/>
@@ -12537,12 +12550,12 @@
         <v>0</v>
       </c>
       <c r="H53" s="3">
-        <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.2</v>
+        <f t="shared" ref="H53:I53" si="4">SUM(H3:H52)</f>
+        <v>0.38</v>
       </c>
       <c r="I53" s="3">
-        <f t="shared" si="3"/>
-        <v>0.02</v>
+        <f t="shared" si="4"/>
+        <v>0.04</v>
       </c>
     </row>
   </sheetData>
@@ -12717,11 +12730,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.45</v>
+        <v>0.66</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -12792,15 +12805,25 @@
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="6"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="17" t="str">
+      <c r="D5" s="10">
+        <v>46231</v>
+      </c>
+      <c r="E5" s="10">
+        <v>46231</v>
+      </c>
+      <c r="F5" s="17">
         <f t="shared" ref="F5:F52" si="0">IF(E5&gt;0,E5-D5,"")</f>
-        <v/>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+        <v>0</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0.21</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0.02</v>
+      </c>
       <c r="J5" s="9"/>
       <c r="X5" s="6">
         <f t="shared" ref="X5:X52" si="1">E4</f>
@@ -12826,11 +12849,11 @@
       <c r="J6" s="9"/>
       <c r="X6" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46231</v>
       </c>
       <c r="Y6" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
@@ -12966,7 +12989,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -13830,11 +13853,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.45</v>
+        <v>0.66</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
     </row>
   </sheetData>
@@ -14009,11 +14032,11 @@
       </c>
       <c r="L3" s="3">
         <f>H53</f>
-        <v>0.94</v>
+        <v>1.23</v>
       </c>
       <c r="M3" s="3">
         <f>I53</f>
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="N3" s="7" t="str">
         <f>IF(B16=K3,XIRR(Y3:Y52,X3:X52),"")</f>
@@ -14115,15 +14138,25 @@
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="2"/>
+      <c r="D6" s="10">
+        <v>46211</v>
+      </c>
+      <c r="E6" s="10">
+        <v>46211</v>
+      </c>
+      <c r="F6" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0.03</v>
+      </c>
       <c r="J6" s="9"/>
       <c r="X6" s="6">
         <f t="shared" si="1"/>
@@ -14149,11 +14182,11 @@
       <c r="J7" s="14"/>
       <c r="X7" s="6">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>46211</v>
       </c>
       <c r="Y7" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
@@ -14267,7 +14300,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>978</v>
+        <v>973</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -15131,11 +15164,11 @@
       </c>
       <c r="H53" s="3">
         <f t="shared" ref="H53:I53" si="3">SUM(H3:H52)</f>
-        <v>0.94</v>
+        <v>1.23</v>
       </c>
       <c r="I53" s="3">
         <f t="shared" si="3"/>
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
     </row>
   </sheetData>
@@ -15589,7 +15622,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -16911,7 +16944,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>
@@ -18253,7 +18286,7 @@
       </c>
       <c r="B12" s="17">
         <f ca="1">IF(B16&lt;&gt;K3,(TODAY()-B11)*-1,"")</f>
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="6"/>

</xml_diff>